<commit_message>
Fix(UI): Corretto ordinamento Timbrature, Refactor Layout Dipendenti e Allineamento Contatori
</commit_message>
<xml_diff>
--- a/Autorizzati ISAB.xlsx
+++ b/Autorizzati ISAB.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luca Riccio\Desktop\CANTIERE ISAB SUD\RISORSE UMANE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Coemi\Desktop\SCRIPT\ISAB_TimeSheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C5DCE9B-EA98-43DA-B74C-98316D38D8CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AFB5E3A-6188-41F8-922C-0715B0273E9D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12570" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Autorizzati ISAB" sheetId="1" r:id="rId1"/>
@@ -22,15 +22,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1432,19 +1423,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I145"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.109375" customWidth="1"/>
-    <col min="2" max="2" width="19.77734375" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" customWidth="1"/>
-    <col min="6" max="6" width="19.77734375" customWidth="1"/>
-    <col min="7" max="8" width="20.77734375" customWidth="1"/>
+    <col min="1" max="1" width="4.140625" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="19.7109375" customWidth="1"/>
+    <col min="7" max="8" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="25.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>248</v>
       </c>
@@ -1471,7 +1463,7 @@
       </c>
       <c r="I1" s="1"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -1498,7 +1490,7 @@
       </c>
       <c r="I2" s="1"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>1</v>
       </c>
@@ -1525,7 +1517,7 @@
       </c>
       <c r="I3" s="1"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
         <v>1</v>
       </c>
@@ -1552,7 +1544,7 @@
       </c>
       <c r="I4" s="1"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="20">
         <v>1</v>
       </c>
@@ -1579,7 +1571,7 @@
       </c>
       <c r="I5" s="1"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="17">
         <v>1</v>
       </c>
@@ -1606,7 +1598,7 @@
       </c>
       <c r="I6" s="1"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="8">
         <v>1</v>
       </c>
@@ -1633,7 +1625,7 @@
       </c>
       <c r="I7" s="1"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
         <v>1</v>
       </c>
@@ -1660,7 +1652,7 @@
       </c>
       <c r="I8" s="1"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="17">
         <v>1</v>
       </c>
@@ -1687,7 +1679,7 @@
       </c>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="17">
         <v>1</v>
       </c>
@@ -1714,7 +1706,7 @@
       </c>
       <c r="I10" s="1"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
         <v>1</v>
       </c>
@@ -1741,7 +1733,7 @@
       </c>
       <c r="I11" s="1"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="17">
         <v>1</v>
       </c>
@@ -1768,7 +1760,7 @@
       </c>
       <c r="I12" s="1"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
         <v>1</v>
       </c>
@@ -1795,7 +1787,7 @@
       </c>
       <c r="I13" s="1"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
         <v>1</v>
       </c>
@@ -1822,7 +1814,7 @@
       </c>
       <c r="I14" s="1"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="17">
         <v>1</v>
       </c>
@@ -1849,7 +1841,7 @@
       </c>
       <c r="I15" s="1"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
         <v>1</v>
       </c>
@@ -1876,7 +1868,7 @@
       </c>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
         <v>1</v>
       </c>
@@ -1903,7 +1895,7 @@
       </c>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
         <v>1</v>
       </c>
@@ -1930,7 +1922,7 @@
       </c>
       <c r="I18" s="1"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
         <v>1</v>
       </c>
@@ -1957,7 +1949,7 @@
       </c>
       <c r="I19" s="1"/>
     </row>
-    <row r="20" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11">
         <v>1</v>
       </c>
@@ -1984,7 +1976,7 @@
       </c>
       <c r="I20" s="3"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
         <v>1</v>
       </c>
@@ -2011,7 +2003,7 @@
       </c>
       <c r="I21" s="1"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
         <v>1</v>
       </c>
@@ -2038,7 +2030,7 @@
       </c>
       <c r="I22" s="1"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
         <v>1</v>
       </c>
@@ -2065,7 +2057,7 @@
       </c>
       <c r="I23" s="1"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8">
         <v>1</v>
       </c>
@@ -2092,7 +2084,7 @@
       </c>
       <c r="I24" s="1"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
         <v>1</v>
       </c>
@@ -2119,7 +2111,7 @@
       </c>
       <c r="I25" s="1"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="17">
         <v>1</v>
       </c>
@@ -2146,7 +2138,7 @@
       </c>
       <c r="I26" s="1"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
         <v>1</v>
       </c>
@@ -2173,7 +2165,7 @@
       </c>
       <c r="I27" s="1"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="8">
         <v>1</v>
       </c>
@@ -2200,7 +2192,7 @@
       </c>
       <c r="I28" s="1"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="8">
         <v>1</v>
       </c>
@@ -2227,7 +2219,7 @@
       </c>
       <c r="I29" s="1"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
         <v>1</v>
       </c>
@@ -2254,7 +2246,7 @@
       </c>
       <c r="I30" s="1"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="8">
         <v>1</v>
       </c>
@@ -2281,7 +2273,7 @@
       </c>
       <c r="I31" s="1"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="17">
         <v>1</v>
       </c>
@@ -2308,7 +2300,7 @@
       </c>
       <c r="I32" s="1"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="8">
         <v>1</v>
       </c>
@@ -2335,7 +2327,7 @@
       </c>
       <c r="I33" s="1"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="17">
         <v>1</v>
       </c>
@@ -2362,7 +2354,7 @@
       </c>
       <c r="I34" s="1"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8">
         <v>1</v>
       </c>
@@ -2389,7 +2381,7 @@
       </c>
       <c r="I35" s="1"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
         <v>1</v>
       </c>
@@ -2416,7 +2408,7 @@
       </c>
       <c r="I36" s="1"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="11">
         <v>1</v>
       </c>
@@ -2443,7 +2435,7 @@
       </c>
       <c r="I37" s="1"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="8">
         <v>1</v>
       </c>
@@ -2470,7 +2462,7 @@
       </c>
       <c r="I38" s="1"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="11">
         <v>1</v>
       </c>
@@ -2497,7 +2489,7 @@
       </c>
       <c r="I39" s="1"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="8">
         <v>1</v>
       </c>
@@ -2524,7 +2516,7 @@
       </c>
       <c r="I40" s="1"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="8">
         <v>1</v>
       </c>
@@ -2551,7 +2543,7 @@
       </c>
       <c r="I41" s="1"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="8">
         <v>1</v>
       </c>
@@ -2578,7 +2570,7 @@
       </c>
       <c r="I42" s="1"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8">
         <v>1</v>
       </c>
@@ -2605,7 +2597,7 @@
       </c>
       <c r="I43" s="1"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="8">
         <v>1</v>
       </c>
@@ -2632,7 +2624,7 @@
       </c>
       <c r="I44" s="1"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="8">
         <v>1</v>
       </c>
@@ -2659,7 +2651,7 @@
       </c>
       <c r="I45" s="1"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="8">
         <v>1</v>
       </c>
@@ -2686,7 +2678,7 @@
       </c>
       <c r="I46" s="1"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
         <v>1</v>
       </c>
@@ -2713,7 +2705,7 @@
       </c>
       <c r="I47" s="1"/>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="17">
         <v>1</v>
       </c>
@@ -2740,7 +2732,7 @@
       </c>
       <c r="I48" s="1"/>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="8">
         <v>1</v>
       </c>
@@ -2767,7 +2759,7 @@
       </c>
       <c r="I49" s="1"/>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="8">
         <v>1</v>
       </c>
@@ -2794,7 +2786,7 @@
       </c>
       <c r="I50" s="1"/>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="8">
         <v>1</v>
       </c>
@@ -2821,7 +2813,7 @@
       </c>
       <c r="I51" s="1"/>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="17">
         <v>1</v>
       </c>
@@ -2848,7 +2840,7 @@
       </c>
       <c r="I52" s="1"/>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="8">
         <v>1</v>
       </c>
@@ -2875,7 +2867,7 @@
       </c>
       <c r="I53" s="1"/>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="8">
         <v>1</v>
       </c>
@@ -2902,7 +2894,7 @@
       </c>
       <c r="I54" s="1"/>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="8">
         <v>1</v>
       </c>
@@ -2929,7 +2921,7 @@
       </c>
       <c r="I55" s="1"/>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="8">
         <v>1</v>
       </c>
@@ -2956,7 +2948,7 @@
       </c>
       <c r="I56" s="1"/>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
         <v>1</v>
       </c>
@@ -2983,7 +2975,7 @@
       </c>
       <c r="I57" s="1"/>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="17">
         <v>1</v>
       </c>
@@ -3010,7 +3002,7 @@
       </c>
       <c r="I58" s="1"/>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="8">
         <v>1</v>
       </c>
@@ -3037,7 +3029,7 @@
       </c>
       <c r="I59" s="1"/>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8">
         <v>1</v>
       </c>
@@ -3064,7 +3056,7 @@
       </c>
       <c r="I60" s="1"/>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="17">
         <v>1</v>
       </c>
@@ -3091,7 +3083,7 @@
       </c>
       <c r="I61" s="1"/>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="17">
         <v>1</v>
       </c>
@@ -3118,7 +3110,7 @@
       </c>
       <c r="I62" s="1"/>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="17">
         <v>1</v>
       </c>
@@ -3145,7 +3137,7 @@
       </c>
       <c r="I63" s="1"/>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="8">
         <v>1</v>
       </c>
@@ -3172,7 +3164,7 @@
       </c>
       <c r="I64" s="1"/>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="8">
         <v>1</v>
       </c>
@@ -3199,7 +3191,7 @@
       </c>
       <c r="I65" s="1"/>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="8">
         <v>1</v>
       </c>
@@ -3226,7 +3218,7 @@
       </c>
       <c r="I66" s="1"/>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="8">
         <v>1</v>
       </c>
@@ -3253,7 +3245,7 @@
       </c>
       <c r="I67" s="1"/>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="8">
         <v>1</v>
       </c>
@@ -3280,7 +3272,7 @@
       </c>
       <c r="I68" s="1"/>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="11">
         <v>1</v>
       </c>
@@ -3307,7 +3299,7 @@
       </c>
       <c r="I69" s="1"/>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="8">
         <v>1</v>
       </c>
@@ -3334,7 +3326,7 @@
       </c>
       <c r="I70" s="1"/>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="17">
         <v>1</v>
       </c>
@@ -3361,7 +3353,7 @@
       </c>
       <c r="I71" s="1"/>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="17">
         <v>1</v>
       </c>
@@ -3388,7 +3380,7 @@
       </c>
       <c r="I72" s="1"/>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="8">
         <v>1</v>
       </c>
@@ -3415,7 +3407,7 @@
       </c>
       <c r="I73" s="1"/>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="8">
         <v>1</v>
       </c>
@@ -3442,7 +3434,7 @@
       </c>
       <c r="I74" s="1"/>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="8">
         <v>1</v>
       </c>
@@ -3469,7 +3461,7 @@
       </c>
       <c r="I75" s="1"/>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="8">
         <v>1</v>
       </c>
@@ -3496,7 +3488,7 @@
       </c>
       <c r="I76" s="1"/>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="17">
         <v>1</v>
       </c>
@@ -3523,7 +3515,7 @@
       </c>
       <c r="I77" s="1"/>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="8">
         <v>1</v>
       </c>
@@ -3550,7 +3542,7 @@
       </c>
       <c r="I78" s="1"/>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="17">
         <v>1</v>
       </c>
@@ -3577,7 +3569,7 @@
       </c>
       <c r="I79" s="1"/>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="8">
         <v>1</v>
       </c>
@@ -3604,7 +3596,7 @@
       </c>
       <c r="I80" s="1"/>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="8">
         <v>1</v>
       </c>
@@ -3631,7 +3623,7 @@
       </c>
       <c r="I81" s="1"/>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="8">
         <v>1</v>
       </c>
@@ -3658,7 +3650,7 @@
       </c>
       <c r="I82" s="1"/>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="8">
         <v>1</v>
       </c>
@@ -3685,7 +3677,7 @@
       </c>
       <c r="I83" s="1"/>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="8">
         <v>1</v>
       </c>
@@ -3712,7 +3704,7 @@
       </c>
       <c r="I84" s="1"/>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="17">
         <v>1</v>
       </c>
@@ -3739,7 +3731,7 @@
       </c>
       <c r="I85" s="1"/>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="8">
         <v>1</v>
       </c>
@@ -3766,7 +3758,7 @@
       </c>
       <c r="I86" s="1"/>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="8">
         <v>1</v>
       </c>
@@ -3793,7 +3785,7 @@
       </c>
       <c r="I87" s="1"/>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="8">
         <v>1</v>
       </c>
@@ -3820,7 +3812,7 @@
       </c>
       <c r="I88" s="1"/>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="8">
         <v>1</v>
       </c>
@@ -3847,7 +3839,7 @@
       </c>
       <c r="I89" s="1"/>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="8">
         <v>1</v>
       </c>
@@ -3874,7 +3866,7 @@
       </c>
       <c r="I90" s="1"/>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="8">
         <v>1</v>
       </c>
@@ -3901,7 +3893,7 @@
       </c>
       <c r="I91" s="1"/>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="8">
         <v>1</v>
       </c>
@@ -3928,7 +3920,7 @@
       </c>
       <c r="I92" s="1"/>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="8">
         <v>1</v>
       </c>
@@ -3955,7 +3947,7 @@
       </c>
       <c r="I93" s="1"/>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="8">
         <v>1</v>
       </c>
@@ -3982,7 +3974,7 @@
       </c>
       <c r="I94" s="1"/>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="8">
         <v>1</v>
       </c>
@@ -4009,7 +4001,7 @@
       </c>
       <c r="I95" s="1"/>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="8">
         <v>1</v>
       </c>
@@ -4036,7 +4028,7 @@
       </c>
       <c r="I96" s="1"/>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="8">
         <v>1</v>
       </c>
@@ -4063,7 +4055,7 @@
       </c>
       <c r="I97" s="1"/>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="8">
         <v>1</v>
       </c>
@@ -4090,7 +4082,7 @@
       </c>
       <c r="I98" s="1"/>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="8">
         <v>1</v>
       </c>
@@ -4117,7 +4109,7 @@
       </c>
       <c r="I99" s="1"/>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="8">
         <v>1</v>
       </c>
@@ -4144,7 +4136,7 @@
       </c>
       <c r="I100" s="1"/>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="8">
         <v>1</v>
       </c>
@@ -4171,7 +4163,7 @@
       </c>
       <c r="I101" s="1"/>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="8">
         <v>1</v>
       </c>
@@ -4198,7 +4190,7 @@
       </c>
       <c r="I102" s="1"/>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="8">
         <v>1</v>
       </c>
@@ -4225,7 +4217,7 @@
       </c>
       <c r="I103" s="1"/>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="17">
         <v>1</v>
       </c>
@@ -4252,7 +4244,7 @@
       </c>
       <c r="I104" s="1"/>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" s="17">
         <v>1</v>
       </c>
@@ -4279,7 +4271,7 @@
       </c>
       <c r="I105" s="1"/>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="8">
         <v>1</v>
       </c>
@@ -4306,7 +4298,7 @@
       </c>
       <c r="I106" s="1"/>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="8">
         <v>1</v>
       </c>
@@ -4333,7 +4325,7 @@
       </c>
       <c r="I107" s="1"/>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="8">
         <v>1</v>
       </c>
@@ -4360,7 +4352,7 @@
       </c>
       <c r="I108" s="1"/>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" s="8">
         <v>1</v>
       </c>
@@ -4387,7 +4379,7 @@
       </c>
       <c r="I109" s="1"/>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" s="8">
         <v>1</v>
       </c>
@@ -4414,7 +4406,7 @@
       </c>
       <c r="I110" s="1"/>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="8">
         <v>1</v>
       </c>
@@ -4441,7 +4433,7 @@
       </c>
       <c r="I111" s="1"/>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="8">
         <v>1</v>
       </c>
@@ -4468,7 +4460,7 @@
       </c>
       <c r="I112" s="1"/>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" s="8">
         <v>1</v>
       </c>
@@ -4495,7 +4487,7 @@
       </c>
       <c r="I113" s="1"/>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" s="17">
         <v>1</v>
       </c>
@@ -4522,10 +4514,10 @@
       </c>
       <c r="I114" s="1"/>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="7">
         <f>SUBTOTAL(9,A2:A114)</f>
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="B115" s="7"/>
       <c r="C115" s="7"/>
@@ -4535,56 +4527,62 @@
       <c r="G115" s="7"/>
       <c r="H115" s="7"/>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138">
         <f>SUBTOTAL(9,A2:A137)</f>
-        <v>113</v>
-      </c>
-    </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A139">
         <f>SUBTOTAL(9,A3:A113)</f>
-        <v>111</v>
-      </c>
-    </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A140">
         <f>SUBTOTAL(9,A2:A139)</f>
-        <v>113</v>
-      </c>
-    </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141">
         <f>SUBTOTAL(9,A3:A113)</f>
-        <v>111</v>
-      </c>
-    </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A142">
         <f>SUBTOTAL(9,A2:A141)</f>
-        <v>113</v>
-      </c>
-    </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A143" s="6">
         <f>SUBTOTAL(9,A3:A113)</f>
-        <v>111</v>
-      </c>
-    </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144">
         <f>SUBTOTAL(9,A2:A143)</f>
-        <v>113</v>
-      </c>
-    </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A145">
         <f>SUBTOTAL(9,A3:A113)</f>
-        <v>111</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H114" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H114" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="7">
+      <filters>
+        <filter val="Valido"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix(OdA): Layout redesign, mapping fix and manual import
</commit_message>
<xml_diff>
--- a/Autorizzati ISAB.xlsx
+++ b/Autorizzati ISAB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Coemi\Desktop\SCRIPT\ISAB_TimeSheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AFB5E3A-6188-41F8-922C-0715B0273E9D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34D7099-2243-4DBF-ADB5-AAD9B4EDF57C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12570" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1076,7 +1076,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1094,7 +1094,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1423,8 +1422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:I145"/>
+  <dimension ref="A1:I144"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" customWidth="1"/>
@@ -1464,3125 +1462,3106 @@
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="17">
-        <v>1</v>
-      </c>
-      <c r="B2" s="18" t="s">
+      <c r="A2" s="16">
+        <v>1</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="19">
+      <c r="D2" s="18">
         <v>34798</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I2" s="1"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="8">
-        <v>1</v>
-      </c>
-      <c r="B3" s="9" t="s">
+      <c r="A3" s="7">
+        <v>1</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>24571</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="9" t="s">
+      <c r="G3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
-        <v>1</v>
-      </c>
-      <c r="B4" s="9" t="s">
+      <c r="A4" s="7">
+        <v>1</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>28202</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="9" t="s">
+      <c r="G4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I4" s="1"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="20">
-        <v>1</v>
-      </c>
-      <c r="B5" s="21" t="s">
+      <c r="A5" s="19">
+        <v>1</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="D5" s="22">
+      <c r="D5" s="21">
         <v>32827</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="E5" s="20" t="s">
         <v>265</v>
       </c>
-      <c r="F5" s="21" t="s">
+      <c r="F5" s="20" t="s">
         <v>276</v>
       </c>
-      <c r="G5" s="21" t="s">
+      <c r="G5" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="H5" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I5" s="1"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="17">
-        <v>1</v>
-      </c>
-      <c r="B6" s="18" t="s">
+      <c r="A6" s="16">
+        <v>1</v>
+      </c>
+      <c r="B6" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="18">
         <v>25238</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="18" t="s">
+      <c r="H6" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="8">
-        <v>1</v>
-      </c>
-      <c r="B7" s="9" t="s">
+      <c r="A7" s="7">
+        <v>1</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="9">
         <v>24908</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="G7" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" s="9" t="s">
+      <c r="G7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
-        <v>1</v>
-      </c>
-      <c r="B8" s="9" t="s">
+      <c r="A8" s="7">
+        <v>1</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="9">
         <v>24199</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" s="9" t="s">
+      <c r="G8" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I8" s="1"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="17">
-        <v>1</v>
-      </c>
-      <c r="B9" s="18" t="s">
+      <c r="A9" s="16">
+        <v>1</v>
+      </c>
+      <c r="B9" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="18">
         <v>27662</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="G9" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="18" t="s">
+      <c r="H9" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I9" s="1"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="17">
-        <v>1</v>
-      </c>
-      <c r="B10" s="18" t="s">
+      <c r="A10" s="16">
+        <v>1</v>
+      </c>
+      <c r="B10" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="18">
         <v>28635</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H10" s="18" t="s">
+      <c r="H10" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="8">
-        <v>1</v>
-      </c>
-      <c r="B11" s="9" t="s">
+      <c r="A11" s="7">
+        <v>1</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="9">
         <v>23389</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="G11" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H11" s="9" t="s">
+      <c r="G11" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I11" s="1"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="17">
-        <v>1</v>
-      </c>
-      <c r="B12" s="18" t="s">
+      <c r="A12" s="16">
+        <v>1</v>
+      </c>
+      <c r="B12" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="18">
         <v>25734</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="G12" s="18" t="s">
+      <c r="G12" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H12" s="18" t="s">
+      <c r="H12" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I12" s="1"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="8">
-        <v>1</v>
-      </c>
-      <c r="B13" s="9" t="s">
+      <c r="A13" s="7">
+        <v>1</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="9">
         <v>28275</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="G13" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H13" s="9" t="s">
+      <c r="G13" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="8">
-        <v>1</v>
-      </c>
-      <c r="B14" s="9" t="s">
+      <c r="A14" s="7">
+        <v>1</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="9">
         <v>37194</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="G14" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H14" s="9" t="s">
+      <c r="G14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H14" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I14" s="1"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="17">
-        <v>1</v>
-      </c>
-      <c r="B15" s="18" t="s">
+      <c r="A15" s="16">
+        <v>1</v>
+      </c>
+      <c r="B15" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="D15" s="19">
+      <c r="D15" s="18">
         <v>32066</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="E15" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="F15" s="18" t="s">
+      <c r="F15" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="G15" s="18" t="s">
+      <c r="G15" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H15" s="18" t="s">
+      <c r="H15" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I15" s="1"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="8">
-        <v>1</v>
-      </c>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="7">
+        <v>1</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="8" t="s">
         <v>246</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="9">
         <v>23043</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="G16" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H16" s="9" t="s">
+      <c r="G16" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I16" s="1"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="8">
-        <v>1</v>
-      </c>
-      <c r="B17" s="9" t="s">
+      <c r="A17" s="7">
+        <v>1</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="9">
         <v>25702</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="G17" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H17" s="9" t="s">
+      <c r="G17" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H17" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="8">
-        <v>1</v>
-      </c>
-      <c r="B18" s="9" t="s">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="7">
+        <v>1</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="9">
         <v>28954</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="E18" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G18" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H18" s="9" t="s">
+      <c r="G18" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H18" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="8">
-        <v>1</v>
-      </c>
-      <c r="B19" s="9" t="s">
+      <c r="A19" s="7">
+        <v>1</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <v>20934</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="G19" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H19" s="9" t="s">
+      <c r="G19" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="11">
-        <v>1</v>
-      </c>
-      <c r="B20" s="12" t="s">
+      <c r="A20" s="10">
+        <v>1</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="D20" s="13">
+      <c r="D20" s="12">
         <v>37579</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="G20" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="H20" s="9" t="s">
+      <c r="G20" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I20" s="3"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="8">
-        <v>1</v>
-      </c>
-      <c r="B21" s="9" t="s">
+      <c r="A21" s="7">
+        <v>1</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="D21" s="10">
+      <c r="D21" s="9">
         <v>21758</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F21" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="G21" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H21" s="9" t="s">
+      <c r="G21" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H21" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="8">
-        <v>1</v>
-      </c>
-      <c r="B22" s="9" t="s">
+      <c r="A22" s="7">
+        <v>1</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D22" s="10">
+      <c r="D22" s="9">
         <v>30682</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F22" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="G22" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H22" s="9" t="s">
+      <c r="G22" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H22" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="11">
-        <v>1</v>
-      </c>
-      <c r="B23" s="12" t="s">
+      <c r="A23" s="10">
+        <v>1</v>
+      </c>
+      <c r="B23" s="11" t="s">
         <v>260</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="C23" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="12">
         <v>30148</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="E23" s="11" t="s">
         <v>252</v>
       </c>
-      <c r="F23" s="12" t="s">
+      <c r="F23" s="11" t="s">
         <v>261</v>
       </c>
-      <c r="G23" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="H23" s="9" t="s">
+      <c r="G23" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H23" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I23" s="1"/>
     </row>
-    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="8">
-        <v>1</v>
-      </c>
-      <c r="B24" s="9" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="7">
+        <v>1</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="9">
         <v>28929</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="F24" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="G24" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H24" s="9" t="s">
+      <c r="G24" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H24" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="8">
-        <v>1</v>
-      </c>
-      <c r="B25" s="9" t="s">
+      <c r="A25" s="7">
+        <v>1</v>
+      </c>
+      <c r="B25" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="9">
         <v>32167</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="F25" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="G25" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H25" s="9" t="s">
+      <c r="G25" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H25" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="17">
-        <v>1</v>
-      </c>
-      <c r="B26" s="18" t="s">
+      <c r="A26" s="16">
+        <v>1</v>
+      </c>
+      <c r="B26" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="C26" s="18" t="s">
+      <c r="C26" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="D26" s="19">
+      <c r="D26" s="18">
         <v>29722</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="E26" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="F26" s="18" t="s">
+      <c r="F26" s="17" t="s">
         <v>254</v>
       </c>
-      <c r="G26" s="23" t="s">
+      <c r="G26" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="H26" s="18" t="s">
+      <c r="H26" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="8">
-        <v>1</v>
-      </c>
-      <c r="B27" s="14" t="s">
+      <c r="A27" s="7">
+        <v>1</v>
+      </c>
+      <c r="B27" s="13" t="s">
         <v>249</v>
       </c>
-      <c r="C27" s="14" t="s">
+      <c r="C27" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="14">
         <v>25292</v>
       </c>
-      <c r="E27" s="14" t="s">
+      <c r="E27" s="13" t="s">
         <v>250</v>
       </c>
-      <c r="F27" s="14" t="s">
+      <c r="F27" s="13" t="s">
         <v>251</v>
       </c>
-      <c r="G27" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H27" s="9" t="s">
+      <c r="G27" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="H27" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="8">
-        <v>1</v>
-      </c>
-      <c r="B28" s="14" t="s">
+      <c r="A28" s="7">
+        <v>1</v>
+      </c>
+      <c r="B28" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="C28" s="14" t="s">
+      <c r="C28" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="15">
+      <c r="D28" s="14">
         <v>25153</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="E28" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="F28" s="14" t="s">
+      <c r="F28" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="G28" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H28" s="9" t="s">
+      <c r="G28" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H28" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="8">
-        <v>1</v>
-      </c>
-      <c r="B29" s="14" t="s">
+      <c r="A29" s="7">
+        <v>1</v>
+      </c>
+      <c r="B29" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="C29" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="D29" s="15">
+      <c r="D29" s="14">
         <v>27297</v>
       </c>
-      <c r="E29" s="14" t="s">
+      <c r="E29" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F29" s="14" t="s">
+      <c r="F29" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="G29" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H29" s="9" t="s">
+      <c r="G29" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H29" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I29" s="1"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="8">
-        <v>1</v>
-      </c>
-      <c r="B30" s="14" t="s">
+      <c r="A30" s="7">
+        <v>1</v>
+      </c>
+      <c r="B30" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="C30" s="14" t="s">
+      <c r="C30" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="14">
         <v>28872</v>
       </c>
-      <c r="E30" s="14" t="s">
+      <c r="E30" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F30" s="14" t="s">
+      <c r="F30" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="G30" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H30" s="9" t="s">
+      <c r="G30" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H30" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="8">
-        <v>1</v>
-      </c>
-      <c r="B31" s="14" t="s">
+      <c r="A31" s="7">
+        <v>1</v>
+      </c>
+      <c r="B31" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="14" t="s">
+      <c r="C31" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="14">
         <v>26462</v>
       </c>
-      <c r="E31" s="14" t="s">
+      <c r="E31" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F31" s="14" t="s">
+      <c r="F31" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="G31" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H31" s="9" t="s">
+      <c r="G31" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H31" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I31" s="1"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="17">
-        <v>1</v>
-      </c>
-      <c r="B32" s="18" t="s">
+      <c r="A32" s="16">
+        <v>1</v>
+      </c>
+      <c r="B32" s="17" t="s">
         <v>255</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C32" s="17" t="s">
         <v>142</v>
       </c>
-      <c r="D32" s="19">
+      <c r="D32" s="18">
         <v>33683</v>
       </c>
-      <c r="E32" s="18" t="s">
+      <c r="E32" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F32" s="18" t="s">
+      <c r="F32" s="17" t="s">
         <v>256</v>
       </c>
-      <c r="G32" s="18" t="s">
+      <c r="G32" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H32" s="18" t="s">
+      <c r="H32" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="8">
-        <v>1</v>
-      </c>
-      <c r="B33" s="9" t="s">
+      <c r="A33" s="7">
+        <v>1</v>
+      </c>
+      <c r="B33" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="D33" s="10">
+      <c r="D33" s="9">
         <v>31930</v>
       </c>
-      <c r="E33" s="9" t="s">
+      <c r="E33" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F33" s="9" t="s">
+      <c r="F33" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="G33" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H33" s="9" t="s">
+      <c r="G33" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H33" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I33" s="1"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="17">
-        <v>1</v>
-      </c>
-      <c r="B34" s="18" t="s">
+      <c r="A34" s="16">
+        <v>1</v>
+      </c>
+      <c r="B34" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="C34" s="18" t="s">
+      <c r="C34" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="D34" s="19">
+      <c r="D34" s="18">
         <v>33234</v>
       </c>
-      <c r="E34" s="18" t="s">
+      <c r="E34" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="F34" s="18" t="s">
+      <c r="F34" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="G34" s="18" t="s">
+      <c r="G34" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H34" s="18" t="s">
+      <c r="H34" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I34" s="1"/>
     </row>
-    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="8">
-        <v>1</v>
-      </c>
-      <c r="B35" s="9" t="s">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="7">
+        <v>1</v>
+      </c>
+      <c r="B35" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D35" s="10">
+      <c r="D35" s="9">
         <v>22676</v>
       </c>
-      <c r="E35" s="9" t="s">
+      <c r="E35" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="F35" s="9" t="s">
+      <c r="F35" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="G35" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H35" s="9" t="s">
+      <c r="G35" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H35" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="11">
-        <v>1</v>
-      </c>
-      <c r="B36" s="12" t="s">
+      <c r="A36" s="10">
+        <v>1</v>
+      </c>
+      <c r="B36" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="C36" s="12" t="s">
+      <c r="C36" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="D36" s="13">
+      <c r="D36" s="12">
         <v>30037</v>
       </c>
-      <c r="E36" s="12" t="s">
+      <c r="E36" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="F36" s="12" t="s">
+      <c r="F36" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="G36" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="H36" s="9" t="s">
+      <c r="G36" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H36" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="11">
-        <v>1</v>
-      </c>
-      <c r="B37" s="12" t="s">
+      <c r="A37" s="10">
+        <v>1</v>
+      </c>
+      <c r="B37" s="11" t="s">
         <v>277</v>
       </c>
-      <c r="C37" s="12" t="s">
+      <c r="C37" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="D37" s="13">
+      <c r="D37" s="12">
         <v>23057</v>
       </c>
-      <c r="E37" s="12" t="s">
+      <c r="E37" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="F37" s="12" t="s">
+      <c r="F37" s="11" t="s">
         <v>278</v>
       </c>
-      <c r="G37" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="H37" s="9" t="s">
+      <c r="G37" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H37" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="8">
-        <v>1</v>
-      </c>
-      <c r="B38" s="9" t="s">
+      <c r="A38" s="7">
+        <v>1</v>
+      </c>
+      <c r="B38" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="C38" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D38" s="10">
+      <c r="D38" s="9">
         <v>24429</v>
       </c>
-      <c r="E38" s="9" t="s">
+      <c r="E38" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F38" s="9" t="s">
+      <c r="F38" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G38" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H38" s="9" t="s">
+      <c r="G38" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H38" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I38" s="1"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="11">
-        <v>1</v>
-      </c>
-      <c r="B39" s="12" t="s">
+      <c r="A39" s="10">
+        <v>1</v>
+      </c>
+      <c r="B39" s="11" t="s">
         <v>262</v>
       </c>
-      <c r="C39" s="12" t="s">
+      <c r="C39" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D39" s="13">
+      <c r="D39" s="12">
         <v>30597</v>
       </c>
-      <c r="E39" s="12" t="s">
+      <c r="E39" s="11" t="s">
         <v>264</v>
       </c>
-      <c r="F39" s="12" t="s">
+      <c r="F39" s="11" t="s">
         <v>263</v>
       </c>
-      <c r="G39" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="H39" s="9" t="s">
+      <c r="G39" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H39" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I39" s="1"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="8">
-        <v>1</v>
-      </c>
-      <c r="B40" s="9" t="s">
+      <c r="A40" s="7">
+        <v>1</v>
+      </c>
+      <c r="B40" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="C40" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="D40" s="10">
+      <c r="D40" s="9">
         <v>25496</v>
       </c>
-      <c r="E40" s="9" t="s">
+      <c r="E40" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F40" s="9" t="s">
+      <c r="F40" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="G40" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H40" s="9" t="s">
+      <c r="G40" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H40" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I40" s="1"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="8">
-        <v>1</v>
-      </c>
-      <c r="B41" s="9" t="s">
+      <c r="A41" s="7">
+        <v>1</v>
+      </c>
+      <c r="B41" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C41" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D41" s="10">
+      <c r="D41" s="9">
         <v>27748</v>
       </c>
-      <c r="E41" s="9" t="s">
+      <c r="E41" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F41" s="9" t="s">
+      <c r="F41" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="G41" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H41" s="9" t="s">
+      <c r="G41" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H41" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I41" s="1"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="8">
-        <v>1</v>
-      </c>
-      <c r="B42" s="9" t="s">
+      <c r="A42" s="7">
+        <v>1</v>
+      </c>
+      <c r="B42" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="D42" s="10">
+      <c r="D42" s="9">
         <v>35990</v>
       </c>
-      <c r="E42" s="9" t="s">
+      <c r="E42" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F42" s="9" t="s">
+      <c r="F42" s="8" t="s">
         <v>285</v>
       </c>
-      <c r="G42" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H42" s="9" t="s">
+      <c r="G42" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H42" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I42" s="1"/>
     </row>
-    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="8">
-        <v>1</v>
-      </c>
-      <c r="B43" s="9" t="s">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="7">
+        <v>1</v>
+      </c>
+      <c r="B43" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D43" s="10">
+      <c r="D43" s="9">
         <v>30957</v>
       </c>
-      <c r="E43" s="9" t="s">
+      <c r="E43" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F43" s="9" t="s">
+      <c r="F43" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="G43" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H43" s="9" t="s">
+      <c r="G43" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H43" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I43" s="1"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="8">
-        <v>1</v>
-      </c>
-      <c r="B44" s="9" t="s">
+      <c r="A44" s="7">
+        <v>1</v>
+      </c>
+      <c r="B44" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C44" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="D44" s="10">
+      <c r="D44" s="9">
         <v>29662</v>
       </c>
-      <c r="E44" s="9" t="s">
+      <c r="E44" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F44" s="9" t="s">
+      <c r="F44" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="G44" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H44" s="9" t="s">
+      <c r="G44" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H44" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I44" s="1"/>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="8">
-        <v>1</v>
-      </c>
-      <c r="B45" s="9" t="s">
+      <c r="A45" s="7">
+        <v>1</v>
+      </c>
+      <c r="B45" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="D45" s="10">
+      <c r="D45" s="9">
         <v>30752</v>
       </c>
-      <c r="E45" s="9" t="s">
+      <c r="E45" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="F45" s="9" t="s">
+      <c r="F45" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="G45" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H45" s="9" t="s">
+      <c r="G45" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H45" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I45" s="1"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="8">
-        <v>1</v>
-      </c>
-      <c r="B46" s="9" t="s">
+      <c r="A46" s="7">
+        <v>1</v>
+      </c>
+      <c r="B46" s="8" t="s">
         <v>290</v>
       </c>
-      <c r="C46" s="9" t="s">
+      <c r="C46" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D46" s="10">
+      <c r="D46" s="9">
         <v>26300</v>
       </c>
-      <c r="E46" s="9" t="s">
+      <c r="E46" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="F46" s="9" t="s">
+      <c r="F46" s="8" t="s">
         <v>292</v>
       </c>
-      <c r="G46" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H46" s="9" t="s">
+      <c r="G46" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H46" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I46" s="1"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="8">
-        <v>1</v>
-      </c>
-      <c r="B47" s="9" t="s">
+      <c r="A47" s="7">
+        <v>1</v>
+      </c>
+      <c r="B47" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="C47" s="9" t="s">
+      <c r="C47" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="D47" s="10">
+      <c r="D47" s="9">
         <v>33263</v>
       </c>
-      <c r="E47" s="9" t="s">
+      <c r="E47" s="8" t="s">
         <v>296</v>
       </c>
-      <c r="F47" s="9" t="s">
+      <c r="F47" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="G47" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H47" s="9" t="s">
+      <c r="G47" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H47" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I47" s="1"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="17">
-        <v>1</v>
-      </c>
-      <c r="B48" s="18" t="s">
+      <c r="A48" s="16">
+        <v>1</v>
+      </c>
+      <c r="B48" s="17" t="s">
         <v>293</v>
       </c>
-      <c r="C48" s="18" t="s">
+      <c r="C48" s="17" t="s">
         <v>294</v>
       </c>
-      <c r="D48" s="19">
+      <c r="D48" s="18">
         <v>26391</v>
       </c>
-      <c r="E48" s="18" t="s">
+      <c r="E48" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F48" s="18" t="s">
+      <c r="F48" s="17" t="s">
         <v>295</v>
       </c>
-      <c r="G48" s="18" t="s">
+      <c r="G48" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H48" s="18" t="s">
+      <c r="H48" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I48" s="1"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="8">
-        <v>1</v>
-      </c>
-      <c r="B49" s="9" t="s">
+      <c r="A49" s="7">
+        <v>1</v>
+      </c>
+      <c r="B49" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="D49" s="10">
+      <c r="D49" s="9">
         <v>24515</v>
       </c>
-      <c r="E49" s="9" t="s">
+      <c r="E49" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="F49" s="9" t="s">
+      <c r="F49" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="G49" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H49" s="9" t="s">
+      <c r="G49" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H49" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I49" s="1"/>
     </row>
-    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="8">
-        <v>1</v>
-      </c>
-      <c r="B50" s="9" t="s">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="7">
+        <v>1</v>
+      </c>
+      <c r="B50" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="C50" s="9" t="s">
+      <c r="C50" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D50" s="10">
+      <c r="D50" s="9">
         <v>29921</v>
       </c>
-      <c r="E50" s="9" t="s">
+      <c r="E50" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F50" s="9" t="s">
+      <c r="F50" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G50" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H50" s="9" t="s">
+      <c r="G50" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H50" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I50" s="1"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" s="8">
-        <v>1</v>
-      </c>
-      <c r="B51" s="9" t="s">
+      <c r="A51" s="7">
+        <v>1</v>
+      </c>
+      <c r="B51" s="8" t="s">
         <v>311</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="C51" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D51" s="10">
+      <c r="D51" s="9">
         <v>25219</v>
       </c>
-      <c r="E51" s="9" t="s">
+      <c r="E51" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="F51" s="9" t="s">
+      <c r="F51" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="G51" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H51" s="9" t="s">
+      <c r="G51" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H51" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I51" s="1"/>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="17">
-        <v>1</v>
-      </c>
-      <c r="B52" s="18" t="s">
+      <c r="A52" s="16">
+        <v>1</v>
+      </c>
+      <c r="B52" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="C52" s="18" t="s">
+      <c r="C52" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="D52" s="19">
+      <c r="D52" s="18">
         <v>33491</v>
       </c>
-      <c r="E52" s="18" t="s">
+      <c r="E52" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F52" s="18" t="s">
+      <c r="F52" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="G52" s="18" t="s">
+      <c r="G52" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H52" s="18" t="s">
+      <c r="H52" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I52" s="1"/>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" s="8">
-        <v>1</v>
-      </c>
-      <c r="B53" s="9" t="s">
+      <c r="A53" s="7">
+        <v>1</v>
+      </c>
+      <c r="B53" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C53" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D53" s="10">
+      <c r="D53" s="9">
         <v>24546</v>
       </c>
-      <c r="E53" s="9" t="s">
+      <c r="E53" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="F53" s="9" t="s">
+      <c r="F53" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="G53" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H53" s="9" t="s">
+      <c r="G53" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H53" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I53" s="1"/>
     </row>
-    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="8">
-        <v>1</v>
-      </c>
-      <c r="B54" s="9" t="s">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="7">
+        <v>1</v>
+      </c>
+      <c r="B54" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="C54" s="9" t="s">
+      <c r="C54" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="D54" s="10">
+      <c r="D54" s="9">
         <v>32917</v>
       </c>
-      <c r="E54" s="9" t="s">
+      <c r="E54" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F54" s="9" t="s">
+      <c r="F54" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="G54" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H54" s="9" t="s">
+      <c r="G54" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H54" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I54" s="1"/>
     </row>
-    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="8">
-        <v>1</v>
-      </c>
-      <c r="B55" s="9" t="s">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" s="7">
+        <v>1</v>
+      </c>
+      <c r="B55" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="C55" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D55" s="10">
+      <c r="D55" s="9">
         <v>22273</v>
       </c>
-      <c r="E55" s="9" t="s">
+      <c r="E55" s="8" t="s">
         <v>297</v>
       </c>
-      <c r="F55" s="9" t="s">
+      <c r="F55" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="G55" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H55" s="9" t="s">
+      <c r="G55" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H55" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I55" s="1"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A56" s="8">
-        <v>1</v>
-      </c>
-      <c r="B56" s="14" t="s">
+      <c r="A56" s="7">
+        <v>1</v>
+      </c>
+      <c r="B56" s="13" t="s">
         <v>281</v>
       </c>
-      <c r="C56" s="14" t="s">
+      <c r="C56" s="13" t="s">
         <v>282</v>
       </c>
-      <c r="D56" s="15">
+      <c r="D56" s="14">
         <v>34632</v>
       </c>
-      <c r="E56" s="14" t="s">
+      <c r="E56" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="F56" s="14" t="s">
+      <c r="F56" s="13" t="s">
         <v>283</v>
       </c>
-      <c r="G56" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H56" s="9" t="s">
+      <c r="G56" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H56" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I56" s="1"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A57" s="8">
-        <v>1</v>
-      </c>
-      <c r="B57" s="9" t="s">
+      <c r="A57" s="7">
+        <v>1</v>
+      </c>
+      <c r="B57" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="C57" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="D57" s="10">
+      <c r="D57" s="9">
         <v>24870</v>
       </c>
-      <c r="E57" s="9" t="s">
+      <c r="E57" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F57" s="9" t="s">
+      <c r="F57" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="G57" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H57" s="9" t="s">
+      <c r="G57" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H57" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I57" s="1"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A58" s="17">
-        <v>1</v>
-      </c>
-      <c r="B58" s="18" t="s">
+      <c r="A58" s="16">
+        <v>1</v>
+      </c>
+      <c r="B58" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="C58" s="18" t="s">
+      <c r="C58" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D58" s="19">
+      <c r="D58" s="18">
         <v>30884</v>
       </c>
-      <c r="E58" s="18" t="s">
+      <c r="E58" s="17" t="s">
         <v>298</v>
       </c>
-      <c r="F58" s="18" t="s">
+      <c r="F58" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="G58" s="18" t="s">
+      <c r="G58" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H58" s="18" t="s">
+      <c r="H58" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I58" s="1"/>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="8">
-        <v>1</v>
-      </c>
-      <c r="B59" s="9" t="s">
+      <c r="A59" s="7">
+        <v>1</v>
+      </c>
+      <c r="B59" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="C59" s="9" t="s">
+      <c r="C59" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="D59" s="10">
+      <c r="D59" s="9">
         <v>29283</v>
       </c>
-      <c r="E59" s="9" t="s">
+      <c r="E59" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F59" s="9" t="s">
+      <c r="F59" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="G59" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H59" s="9" t="s">
+      <c r="G59" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H59" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I59" s="1"/>
     </row>
-    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="8">
-        <v>1</v>
-      </c>
-      <c r="B60" s="9" t="s">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" s="7">
+        <v>1</v>
+      </c>
+      <c r="B60" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="C60" s="9" t="s">
+      <c r="C60" s="8" t="s">
         <v>270</v>
       </c>
-      <c r="D60" s="10">
+      <c r="D60" s="9">
         <v>31531</v>
       </c>
-      <c r="E60" s="9" t="s">
+      <c r="E60" s="8" t="s">
         <v>299</v>
       </c>
-      <c r="F60" s="9" t="s">
+      <c r="F60" s="8" t="s">
         <v>271</v>
       </c>
-      <c r="G60" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H60" s="9" t="s">
+      <c r="G60" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H60" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I60" s="1"/>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A61" s="17">
-        <v>1</v>
-      </c>
-      <c r="B61" s="18" t="s">
+      <c r="A61" s="16">
+        <v>1</v>
+      </c>
+      <c r="B61" s="17" t="s">
         <v>138</v>
       </c>
-      <c r="C61" s="18" t="s">
+      <c r="C61" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="D61" s="19">
+      <c r="D61" s="18">
         <v>26155</v>
       </c>
-      <c r="E61" s="18" t="s">
+      <c r="E61" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F61" s="18" t="s">
+      <c r="F61" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="G61" s="18" t="s">
+      <c r="G61" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H61" s="18" t="s">
+      <c r="H61" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I61" s="1"/>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" s="17">
-        <v>1</v>
-      </c>
-      <c r="B62" s="18" t="s">
+      <c r="A62" s="16">
+        <v>1</v>
+      </c>
+      <c r="B62" s="17" t="s">
         <v>272</v>
       </c>
-      <c r="C62" s="18" t="s">
+      <c r="C62" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D62" s="19">
+      <c r="D62" s="18">
         <v>27479</v>
       </c>
-      <c r="E62" s="18" t="s">
+      <c r="E62" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="F62" s="18" t="s">
+      <c r="F62" s="17" t="s">
         <v>273</v>
       </c>
-      <c r="G62" s="18" t="s">
+      <c r="G62" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H62" s="18" t="s">
+      <c r="H62" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I62" s="1"/>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A63" s="17">
-        <v>1</v>
-      </c>
-      <c r="B63" s="18" t="s">
+      <c r="A63" s="16">
+        <v>1</v>
+      </c>
+      <c r="B63" s="17" t="s">
         <v>257</v>
       </c>
-      <c r="C63" s="18" t="s">
+      <c r="C63" s="17" t="s">
         <v>258</v>
       </c>
-      <c r="D63" s="19">
+      <c r="D63" s="18">
         <v>26048</v>
       </c>
-      <c r="E63" s="18" t="s">
+      <c r="E63" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="F63" s="18" t="s">
+      <c r="F63" s="17" t="s">
         <v>259</v>
       </c>
-      <c r="G63" s="18" t="s">
+      <c r="G63" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H63" s="18" t="s">
+      <c r="H63" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I63" s="1"/>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A64" s="8">
-        <v>1</v>
-      </c>
-      <c r="B64" s="9" t="s">
+      <c r="A64" s="7">
+        <v>1</v>
+      </c>
+      <c r="B64" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="C64" s="9" t="s">
+      <c r="C64" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="D64" s="10">
+      <c r="D64" s="9">
         <v>25660</v>
       </c>
-      <c r="E64" s="9" t="s">
+      <c r="E64" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="F64" s="9" t="s">
+      <c r="F64" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="G64" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H64" s="9" t="s">
+      <c r="G64" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H64" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I64" s="1"/>
     </row>
-    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="8">
-        <v>1</v>
-      </c>
-      <c r="B65" s="9" t="s">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65" s="7">
+        <v>1</v>
+      </c>
+      <c r="B65" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="C65" s="9" t="s">
+      <c r="C65" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="D65" s="10">
+      <c r="D65" s="9">
         <v>37477</v>
       </c>
-      <c r="E65" s="9" t="s">
+      <c r="E65" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F65" s="9" t="s">
+      <c r="F65" s="8" t="s">
         <v>307</v>
       </c>
-      <c r="G65" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H65" s="9" t="s">
+      <c r="G65" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H65" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I65" s="1"/>
     </row>
-    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="8">
-        <v>1</v>
-      </c>
-      <c r="B66" s="9" t="s">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" s="7">
+        <v>1</v>
+      </c>
+      <c r="B66" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="C66" s="9" t="s">
+      <c r="C66" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="D66" s="10">
+      <c r="D66" s="9">
         <v>30946</v>
       </c>
-      <c r="E66" s="9" t="s">
+      <c r="E66" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F66" s="9" t="s">
+      <c r="F66" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="G66" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H66" s="9" t="s">
+      <c r="G66" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H66" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I66" s="1"/>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A67" s="8">
-        <v>1</v>
-      </c>
-      <c r="B67" s="9" t="s">
+      <c r="A67" s="7">
+        <v>1</v>
+      </c>
+      <c r="B67" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C67" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D67" s="10">
+      <c r="D67" s="9">
         <v>26998</v>
       </c>
-      <c r="E67" s="9" t="s">
+      <c r="E67" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F67" s="9" t="s">
+      <c r="F67" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="G67" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H67" s="9" t="s">
+      <c r="G67" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H67" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I67" s="1"/>
     </row>
-    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="8">
-        <v>1</v>
-      </c>
-      <c r="B68" s="9" t="s">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68" s="7">
+        <v>1</v>
+      </c>
+      <c r="B68" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="C68" s="9" t="s">
+      <c r="C68" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="D68" s="10">
+      <c r="D68" s="9">
         <v>28358</v>
       </c>
-      <c r="E68" s="9" t="s">
+      <c r="E68" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="F68" s="9" t="s">
+      <c r="F68" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="G68" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H68" s="9" t="s">
+      <c r="G68" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H68" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I68" s="1"/>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A69" s="11">
-        <v>1</v>
-      </c>
-      <c r="B69" s="12" t="s">
+      <c r="A69" s="10">
+        <v>1</v>
+      </c>
+      <c r="B69" s="11" t="s">
         <v>266</v>
       </c>
-      <c r="C69" s="12" t="s">
+      <c r="C69" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="D69" s="13">
+      <c r="D69" s="12">
         <v>33066</v>
       </c>
-      <c r="E69" s="12" t="s">
+      <c r="E69" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="F69" s="12" t="s">
+      <c r="F69" s="11" t="s">
         <v>267</v>
       </c>
-      <c r="G69" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="H69" s="9" t="s">
+      <c r="G69" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H69" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I69" s="1"/>
     </row>
-    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="8">
-        <v>1</v>
-      </c>
-      <c r="B70" s="9" t="s">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A70" s="7">
+        <v>1</v>
+      </c>
+      <c r="B70" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="C70" s="9" t="s">
+      <c r="C70" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="D70" s="10">
+      <c r="D70" s="9">
         <v>32743</v>
       </c>
-      <c r="E70" s="9" t="s">
+      <c r="E70" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F70" s="9" t="s">
+      <c r="F70" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="G70" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H70" s="9" t="s">
+      <c r="G70" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H70" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I70" s="1"/>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A71" s="17">
-        <v>1</v>
-      </c>
-      <c r="B71" s="18" t="s">
+      <c r="A71" s="16">
+        <v>1</v>
+      </c>
+      <c r="B71" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="C71" s="18" t="s">
+      <c r="C71" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="D71" s="19">
+      <c r="D71" s="18">
         <v>24784</v>
       </c>
-      <c r="E71" s="18" t="s">
+      <c r="E71" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="F71" s="18" t="s">
+      <c r="F71" s="17" t="s">
         <v>156</v>
       </c>
-      <c r="G71" s="18" t="s">
+      <c r="G71" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H71" s="18" t="s">
+      <c r="H71" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I71" s="1"/>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A72" s="17">
-        <v>1</v>
-      </c>
-      <c r="B72" s="18" t="s">
+      <c r="A72" s="16">
+        <v>1</v>
+      </c>
+      <c r="B72" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="C72" s="18" t="s">
+      <c r="C72" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="D72" s="19">
+      <c r="D72" s="18">
         <v>29518</v>
       </c>
-      <c r="E72" s="18" t="s">
+      <c r="E72" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="F72" s="18" t="s">
+      <c r="F72" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="G72" s="18" t="s">
+      <c r="G72" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H72" s="18" t="s">
+      <c r="H72" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I72" s="1"/>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A73" s="8">
-        <v>1</v>
-      </c>
-      <c r="B73" s="9" t="s">
+      <c r="A73" s="7">
+        <v>1</v>
+      </c>
+      <c r="B73" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C73" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D73" s="10">
+      <c r="D73" s="9">
         <v>33646</v>
       </c>
-      <c r="E73" s="9" t="s">
+      <c r="E73" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F73" s="9" t="s">
+      <c r="F73" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="G73" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H73" s="9" t="s">
+      <c r="G73" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H73" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I73" s="1"/>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A74" s="8">
-        <v>1</v>
-      </c>
-      <c r="B74" s="9" t="s">
+      <c r="A74" s="7">
+        <v>1</v>
+      </c>
+      <c r="B74" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="C74" s="9" t="s">
+      <c r="C74" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="D74" s="10">
+      <c r="D74" s="9">
         <v>23109</v>
       </c>
-      <c r="E74" s="9" t="s">
+      <c r="E74" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="F74" s="9" t="s">
+      <c r="F74" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="G74" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H74" s="9" t="s">
+      <c r="G74" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H74" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I74" s="1"/>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A75" s="8">
-        <v>1</v>
-      </c>
-      <c r="B75" s="9" t="s">
+      <c r="A75" s="7">
+        <v>1</v>
+      </c>
+      <c r="B75" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="C75" s="9" t="s">
+      <c r="C75" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="D75" s="10">
+      <c r="D75" s="9">
         <v>36165</v>
       </c>
-      <c r="E75" s="9" t="s">
+      <c r="E75" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F75" s="9" t="s">
+      <c r="F75" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="G75" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H75" s="9" t="s">
+      <c r="G75" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H75" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I75" s="1"/>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A76" s="8">
-        <v>1</v>
-      </c>
-      <c r="B76" s="9" t="s">
+      <c r="A76" s="7">
+        <v>1</v>
+      </c>
+      <c r="B76" s="8" t="s">
         <v>304</v>
       </c>
-      <c r="C76" s="9" t="s">
+      <c r="C76" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="D76" s="10">
+      <c r="D76" s="9">
         <v>34008</v>
       </c>
-      <c r="E76" s="9" t="s">
+      <c r="E76" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F76" s="9" t="s">
+      <c r="F76" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="G76" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H76" s="9" t="s">
+      <c r="G76" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H76" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I76" s="1"/>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A77" s="17">
-        <v>1</v>
-      </c>
-      <c r="B77" s="18" t="s">
+      <c r="A77" s="16">
+        <v>1</v>
+      </c>
+      <c r="B77" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="C77" s="18" t="s">
+      <c r="C77" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="D77" s="19">
+      <c r="D77" s="18">
         <v>33263</v>
       </c>
-      <c r="E77" s="18" t="s">
+      <c r="E77" s="17" t="s">
         <v>300</v>
       </c>
-      <c r="F77" s="18" t="s">
+      <c r="F77" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="G77" s="18" t="s">
+      <c r="G77" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H77" s="18" t="s">
+      <c r="H77" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I77" s="1"/>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A78" s="8">
-        <v>1</v>
-      </c>
-      <c r="B78" s="9" t="s">
+      <c r="A78" s="7">
+        <v>1</v>
+      </c>
+      <c r="B78" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="C78" s="9" t="s">
+      <c r="C78" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D78" s="10">
+      <c r="D78" s="9">
         <v>23043</v>
       </c>
-      <c r="E78" s="9" t="s">
+      <c r="E78" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="F78" s="9" t="s">
+      <c r="F78" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="G78" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H78" s="9" t="s">
+      <c r="G78" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H78" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I78" s="1"/>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A79" s="17">
-        <v>1</v>
-      </c>
-      <c r="B79" s="18" t="s">
+      <c r="A79" s="16">
+        <v>1</v>
+      </c>
+      <c r="B79" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="C79" s="18" t="s">
+      <c r="C79" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="D79" s="19">
+      <c r="D79" s="18">
         <v>19329</v>
       </c>
-      <c r="E79" s="18" t="s">
+      <c r="E79" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="F79" s="18" t="s">
+      <c r="F79" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="G79" s="18" t="s">
+      <c r="G79" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H79" s="18" t="s">
+      <c r="H79" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I79" s="1"/>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A80" s="8">
-        <v>1</v>
-      </c>
-      <c r="B80" s="9" t="s">
+      <c r="A80" s="7">
+        <v>1</v>
+      </c>
+      <c r="B80" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="C80" s="9" t="s">
+      <c r="C80" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D80" s="10">
+      <c r="D80" s="9">
         <v>16502</v>
       </c>
-      <c r="E80" s="9" t="s">
+      <c r="E80" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F80" s="9" t="s">
+      <c r="F80" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="G80" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H80" s="9" t="s">
+      <c r="G80" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H80" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I80" s="1"/>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A81" s="8">
-        <v>1</v>
-      </c>
-      <c r="B81" s="9" t="s">
+      <c r="A81" s="7">
+        <v>1</v>
+      </c>
+      <c r="B81" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="C81" s="9" t="s">
+      <c r="C81" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D81" s="10">
+      <c r="D81" s="9">
         <v>25758</v>
       </c>
-      <c r="E81" s="9" t="s">
+      <c r="E81" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F81" s="9" t="s">
+      <c r="F81" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="G81" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H81" s="9" t="s">
+      <c r="G81" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H81" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I81" s="1"/>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A82" s="8">
-        <v>1</v>
-      </c>
-      <c r="B82" s="9" t="s">
+      <c r="A82" s="7">
+        <v>1</v>
+      </c>
+      <c r="B82" s="8" t="s">
         <v>287</v>
       </c>
-      <c r="C82" s="9" t="s">
+      <c r="C82" s="8" t="s">
         <v>288</v>
       </c>
-      <c r="D82" s="10">
+      <c r="D82" s="9">
         <v>22036</v>
       </c>
-      <c r="E82" s="9" t="s">
+      <c r="E82" s="8" t="s">
         <v>301</v>
       </c>
-      <c r="F82" s="9" t="s">
+      <c r="F82" s="8" t="s">
         <v>289</v>
       </c>
-      <c r="G82" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H82" s="9" t="s">
+      <c r="G82" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H82" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I82" s="1"/>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A83" s="8">
-        <v>1</v>
-      </c>
-      <c r="B83" s="9" t="s">
+      <c r="A83" s="7">
+        <v>1</v>
+      </c>
+      <c r="B83" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="C83" s="9" t="s">
+      <c r="C83" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D83" s="10">
+      <c r="D83" s="9">
         <v>29999</v>
       </c>
-      <c r="E83" s="9" t="s">
+      <c r="E83" s="8" t="s">
         <v>252</v>
       </c>
-      <c r="F83" s="9" t="s">
+      <c r="F83" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="G83" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H83" s="9" t="s">
+      <c r="G83" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H83" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I83" s="1"/>
     </row>
-    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="8">
-        <v>1</v>
-      </c>
-      <c r="B84" s="14" t="s">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A84" s="7">
+        <v>1</v>
+      </c>
+      <c r="B84" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="C84" s="14" t="s">
+      <c r="C84" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="D84" s="15">
+      <c r="D84" s="14">
         <v>34611</v>
       </c>
-      <c r="E84" s="14" t="s">
+      <c r="E84" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="F84" s="14" t="s">
+      <c r="F84" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="G84" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H84" s="9" t="s">
+      <c r="G84" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H84" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I84" s="1"/>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A85" s="17">
-        <v>1</v>
-      </c>
-      <c r="B85" s="18" t="s">
+      <c r="A85" s="16">
+        <v>1</v>
+      </c>
+      <c r="B85" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="C85" s="18" t="s">
+      <c r="C85" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="D85" s="19">
+      <c r="D85" s="18">
         <v>28973</v>
       </c>
-      <c r="E85" s="18" t="s">
+      <c r="E85" s="17" t="s">
         <v>302</v>
       </c>
-      <c r="F85" s="18" t="s">
+      <c r="F85" s="17" t="s">
         <v>180</v>
       </c>
-      <c r="G85" s="18" t="s">
+      <c r="G85" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H85" s="18" t="s">
+      <c r="H85" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I85" s="1"/>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A86" s="8">
-        <v>1</v>
-      </c>
-      <c r="B86" s="14" t="s">
+      <c r="A86" s="7">
+        <v>1</v>
+      </c>
+      <c r="B86" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="C86" s="14" t="s">
+      <c r="C86" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="D86" s="15">
+      <c r="D86" s="14">
         <v>37138</v>
       </c>
-      <c r="E86" s="14" t="s">
+      <c r="E86" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="F86" s="14" t="s">
+      <c r="F86" s="13" t="s">
         <v>286</v>
       </c>
-      <c r="G86" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H86" s="9" t="s">
+      <c r="G86" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H86" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I86" s="1"/>
     </row>
-    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="8">
-        <v>1</v>
-      </c>
-      <c r="B87" s="14" t="s">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A87" s="7">
+        <v>1</v>
+      </c>
+      <c r="B87" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="C87" s="14" t="s">
+      <c r="C87" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="D87" s="15">
+      <c r="D87" s="14">
         <v>35599</v>
       </c>
-      <c r="E87" s="14" t="s">
+      <c r="E87" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="F87" s="14" t="s">
+      <c r="F87" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="G87" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H87" s="9" t="s">
+      <c r="G87" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H87" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I87" s="1"/>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A88" s="8">
-        <v>1</v>
-      </c>
-      <c r="B88" s="14" t="s">
+      <c r="A88" s="7">
+        <v>1</v>
+      </c>
+      <c r="B88" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="C88" s="14" t="s">
+      <c r="C88" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="D88" s="15">
+      <c r="D88" s="14">
         <v>22908</v>
       </c>
-      <c r="E88" s="14" t="s">
+      <c r="E88" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F88" s="14" t="s">
+      <c r="F88" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="G88" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H88" s="9" t="s">
+      <c r="G88" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H88" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I88" s="1"/>
     </row>
-    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="8">
-        <v>1</v>
-      </c>
-      <c r="B89" s="14" t="s">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A89" s="7">
+        <v>1</v>
+      </c>
+      <c r="B89" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="C89" s="14" t="s">
+      <c r="C89" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="D89" s="15">
+      <c r="D89" s="14">
         <v>33883</v>
       </c>
-      <c r="E89" s="14" t="s">
+      <c r="E89" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="F89" s="14" t="s">
+      <c r="F89" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="G89" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H89" s="9" t="s">
+      <c r="G89" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H89" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I89" s="1"/>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A90" s="8">
-        <v>1</v>
-      </c>
-      <c r="B90" s="14" t="s">
+      <c r="A90" s="7">
+        <v>1</v>
+      </c>
+      <c r="B90" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="C90" s="14" t="s">
+      <c r="C90" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="D90" s="15">
+      <c r="D90" s="14">
         <v>30213</v>
       </c>
-      <c r="E90" s="14" t="s">
+      <c r="E90" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="F90" s="14" t="s">
+      <c r="F90" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="G90" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H90" s="9" t="s">
+      <c r="G90" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H90" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I90" s="1"/>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A91" s="8">
-        <v>1</v>
-      </c>
-      <c r="B91" s="14" t="s">
+      <c r="A91" s="7">
+        <v>1</v>
+      </c>
+      <c r="B91" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="C91" s="14" t="s">
+      <c r="C91" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="D91" s="15">
+      <c r="D91" s="14">
         <v>30570</v>
       </c>
-      <c r="E91" s="14" t="s">
+      <c r="E91" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="F91" s="14" t="s">
+      <c r="F91" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="G91" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H91" s="9" t="s">
+      <c r="G91" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H91" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I91" s="1"/>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A92" s="8">
-        <v>1</v>
-      </c>
-      <c r="B92" s="14" t="s">
+      <c r="A92" s="7">
+        <v>1</v>
+      </c>
+      <c r="B92" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="C92" s="14" t="s">
+      <c r="C92" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="D92" s="15">
+      <c r="D92" s="14">
         <v>26258</v>
       </c>
-      <c r="E92" s="14" t="s">
+      <c r="E92" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="F92" s="14" t="s">
+      <c r="F92" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="G92" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H92" s="9" t="s">
+      <c r="G92" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H92" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I92" s="1"/>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A93" s="8">
-        <v>1</v>
-      </c>
-      <c r="B93" s="14" t="s">
+      <c r="A93" s="7">
+        <v>1</v>
+      </c>
+      <c r="B93" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="C93" s="14" t="s">
+      <c r="C93" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="D93" s="15">
+      <c r="D93" s="14">
         <v>28358</v>
       </c>
-      <c r="E93" s="14" t="s">
+      <c r="E93" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F93" s="14" t="s">
+      <c r="F93" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="G93" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H93" s="9" t="s">
+      <c r="G93" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H93" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I93" s="1"/>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A94" s="8">
-        <v>1</v>
-      </c>
-      <c r="B94" s="14" t="s">
+      <c r="A94" s="7">
+        <v>1</v>
+      </c>
+      <c r="B94" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="C94" s="14" t="s">
+      <c r="C94" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="D94" s="15">
+      <c r="D94" s="14">
         <v>29217</v>
       </c>
-      <c r="E94" s="14" t="s">
+      <c r="E94" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="F94" s="14" t="s">
+      <c r="F94" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="G94" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H94" s="9" t="s">
+      <c r="G94" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H94" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I94" s="1"/>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A95" s="8">
-        <v>1</v>
-      </c>
-      <c r="B95" s="14" t="s">
+      <c r="A95" s="7">
+        <v>1</v>
+      </c>
+      <c r="B95" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="C95" s="14" t="s">
+      <c r="C95" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="D95" s="15">
+      <c r="D95" s="14">
         <v>27913</v>
       </c>
-      <c r="E95" s="14" t="s">
+      <c r="E95" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="F95" s="14" t="s">
+      <c r="F95" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="G95" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H95" s="9" t="s">
+      <c r="G95" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H95" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I95" s="1"/>
     </row>
-    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="8">
-        <v>1</v>
-      </c>
-      <c r="B96" s="9" t="s">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A96" s="7">
+        <v>1</v>
+      </c>
+      <c r="B96" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="C96" s="9" t="s">
+      <c r="C96" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="D96" s="10">
+      <c r="D96" s="9">
         <v>30716</v>
       </c>
-      <c r="E96" s="9" t="s">
+      <c r="E96" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F96" s="9" t="s">
+      <c r="F96" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="G96" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H96" s="9" t="s">
+      <c r="G96" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H96" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I96" s="1"/>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A97" s="8">
-        <v>1</v>
-      </c>
-      <c r="B97" s="9" t="s">
+      <c r="A97" s="7">
+        <v>1</v>
+      </c>
+      <c r="B97" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="C97" s="9" t="s">
+      <c r="C97" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D97" s="10">
+      <c r="D97" s="9">
         <v>23817</v>
       </c>
-      <c r="E97" s="9" t="s">
+      <c r="E97" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="F97" s="9" t="s">
+      <c r="F97" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="G97" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H97" s="9" t="s">
+      <c r="G97" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H97" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I97" s="1"/>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A98" s="8">
-        <v>1</v>
-      </c>
-      <c r="B98" s="9" t="s">
+      <c r="A98" s="7">
+        <v>1</v>
+      </c>
+      <c r="B98" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="C98" s="9" t="s">
+      <c r="C98" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D98" s="10">
+      <c r="D98" s="9">
         <v>32361</v>
       </c>
-      <c r="E98" s="9" t="s">
+      <c r="E98" s="8" t="s">
         <v>303</v>
       </c>
-      <c r="F98" s="9" t="s">
+      <c r="F98" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="G98" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H98" s="9" t="s">
+      <c r="G98" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H98" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I98" s="1"/>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A99" s="8">
-        <v>1</v>
-      </c>
-      <c r="B99" s="9" t="s">
+      <c r="A99" s="7">
+        <v>1</v>
+      </c>
+      <c r="B99" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="C99" s="9" t="s">
+      <c r="C99" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="D99" s="10">
+      <c r="D99" s="9">
         <v>26409</v>
       </c>
-      <c r="E99" s="9" t="s">
+      <c r="E99" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="F99" s="9" t="s">
+      <c r="F99" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="G99" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H99" s="9" t="s">
+      <c r="G99" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H99" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I99" s="1"/>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A100" s="8">
-        <v>1</v>
-      </c>
-      <c r="B100" s="9" t="s">
+      <c r="A100" s="7">
+        <v>1</v>
+      </c>
+      <c r="B100" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="C100" s="9" t="s">
+      <c r="C100" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="D100" s="10">
+      <c r="D100" s="9">
         <v>29737</v>
       </c>
-      <c r="E100" s="9" t="s">
+      <c r="E100" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F100" s="9" t="s">
+      <c r="F100" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="G100" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H100" s="9" t="s">
+      <c r="G100" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H100" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I100" s="1"/>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A101" s="8">
-        <v>1</v>
-      </c>
-      <c r="B101" s="9" t="s">
+      <c r="A101" s="7">
+        <v>1</v>
+      </c>
+      <c r="B101" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="C101" s="9" t="s">
+      <c r="C101" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="D101" s="10">
+      <c r="D101" s="9">
         <v>24490</v>
       </c>
-      <c r="E101" s="9" t="s">
+      <c r="E101" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F101" s="9" t="s">
+      <c r="F101" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="G101" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H101" s="9" t="s">
+      <c r="G101" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H101" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I101" s="1"/>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A102" s="8">
-        <v>1</v>
-      </c>
-      <c r="B102" s="9" t="s">
+      <c r="A102" s="7">
+        <v>1</v>
+      </c>
+      <c r="B102" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="C102" s="9" t="s">
+      <c r="C102" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D102" s="10">
+      <c r="D102" s="9">
         <v>32366</v>
       </c>
-      <c r="E102" s="9" t="s">
+      <c r="E102" s="8" t="s">
         <v>220</v>
       </c>
-      <c r="F102" s="9" t="s">
+      <c r="F102" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="G102" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H102" s="9" t="s">
+      <c r="G102" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H102" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I102" s="1"/>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A103" s="8">
-        <v>1</v>
-      </c>
-      <c r="B103" s="9" t="s">
+      <c r="A103" s="7">
+        <v>1</v>
+      </c>
+      <c r="B103" s="8" t="s">
         <v>279</v>
       </c>
-      <c r="C103" s="9" t="s">
+      <c r="C103" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D103" s="10">
+      <c r="D103" s="9">
         <v>38772</v>
       </c>
-      <c r="E103" s="9" t="s">
+      <c r="E103" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F103" s="9" t="s">
+      <c r="F103" s="8" t="s">
         <v>280</v>
       </c>
-      <c r="G103" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H103" s="9" t="s">
+      <c r="G103" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H103" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I103" s="1"/>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A104" s="17">
-        <v>1</v>
-      </c>
-      <c r="B104" s="18" t="s">
+      <c r="A104" s="16">
+        <v>1</v>
+      </c>
+      <c r="B104" s="17" t="s">
         <v>222</v>
       </c>
-      <c r="C104" s="18" t="s">
+      <c r="C104" s="17" t="s">
         <v>223</v>
       </c>
-      <c r="D104" s="19">
+      <c r="D104" s="18">
         <v>22429</v>
       </c>
-      <c r="E104" s="18" t="s">
+      <c r="E104" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F104" s="18" t="s">
+      <c r="F104" s="17" t="s">
         <v>224</v>
       </c>
-      <c r="G104" s="18" t="s">
+      <c r="G104" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H104" s="18" t="s">
+      <c r="H104" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I104" s="1"/>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A105" s="17">
-        <v>1</v>
-      </c>
-      <c r="B105" s="18" t="s">
+      <c r="A105" s="16">
+        <v>1</v>
+      </c>
+      <c r="B105" s="17" t="s">
         <v>225</v>
       </c>
-      <c r="C105" s="18" t="s">
+      <c r="C105" s="17" t="s">
         <v>226</v>
       </c>
-      <c r="D105" s="19">
+      <c r="D105" s="18">
         <v>26675</v>
       </c>
-      <c r="E105" s="18" t="s">
+      <c r="E105" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="F105" s="18" t="s">
+      <c r="F105" s="17" t="s">
         <v>227</v>
       </c>
-      <c r="G105" s="18" t="s">
+      <c r="G105" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H105" s="18" t="s">
+      <c r="H105" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I105" s="1"/>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A106" s="8">
-        <v>1</v>
-      </c>
-      <c r="B106" s="9" t="s">
+      <c r="A106" s="7">
+        <v>1</v>
+      </c>
+      <c r="B106" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="C106" s="9" t="s">
+      <c r="C106" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D106" s="10">
+      <c r="D106" s="9">
         <v>28748</v>
       </c>
-      <c r="E106" s="9" t="s">
+      <c r="E106" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F106" s="9" t="s">
+      <c r="F106" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="G106" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H106" s="9" t="s">
+      <c r="G106" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H106" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I106" s="1"/>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A107" s="8">
-        <v>1</v>
-      </c>
-      <c r="B107" s="9" t="s">
+      <c r="A107" s="7">
+        <v>1</v>
+      </c>
+      <c r="B107" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="C107" s="9" t="s">
+      <c r="C107" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D107" s="10">
+      <c r="D107" s="9">
         <v>22225</v>
       </c>
-      <c r="E107" s="9" t="s">
+      <c r="E107" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F107" s="9" t="s">
+      <c r="F107" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="G107" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H107" s="9" t="s">
+      <c r="G107" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H107" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I107" s="1"/>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A108" s="8">
-        <v>1</v>
-      </c>
-      <c r="B108" s="14" t="s">
+      <c r="A108" s="7">
+        <v>1</v>
+      </c>
+      <c r="B108" s="13" t="s">
         <v>268</v>
       </c>
-      <c r="C108" s="14" t="s">
+      <c r="C108" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="D108" s="15">
+      <c r="D108" s="14">
         <v>38224</v>
       </c>
-      <c r="E108" s="14" t="s">
+      <c r="E108" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="F108" s="14" t="s">
+      <c r="F108" s="13" t="s">
         <v>269</v>
       </c>
-      <c r="G108" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H108" s="9" t="s">
+      <c r="G108" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H108" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I108" s="1"/>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A109" s="8">
-        <v>1</v>
-      </c>
-      <c r="B109" s="9" t="s">
+      <c r="A109" s="7">
+        <v>1</v>
+      </c>
+      <c r="B109" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="C109" s="9" t="s">
+      <c r="C109" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="D109" s="10">
+      <c r="D109" s="9">
         <v>30848</v>
       </c>
-      <c r="E109" s="9" t="s">
+      <c r="E109" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F109" s="9" t="s">
+      <c r="F109" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="G109" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H109" s="9" t="s">
+      <c r="G109" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H109" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I109" s="1"/>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A110" s="8">
-        <v>1</v>
-      </c>
-      <c r="B110" s="9" t="s">
+      <c r="A110" s="7">
+        <v>1</v>
+      </c>
+      <c r="B110" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="C110" s="9" t="s">
+      <c r="C110" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="D110" s="10">
+      <c r="D110" s="9">
         <v>31256</v>
       </c>
-      <c r="E110" s="9" t="s">
+      <c r="E110" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F110" s="9" t="s">
+      <c r="F110" s="8" t="s">
         <v>235</v>
       </c>
-      <c r="G110" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H110" s="9" t="s">
+      <c r="G110" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H110" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I110" s="1"/>
     </row>
-    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="8">
-        <v>1</v>
-      </c>
-      <c r="B111" s="9" t="s">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A111" s="7">
+        <v>1</v>
+      </c>
+      <c r="B111" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="C111" s="9" t="s">
+      <c r="C111" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D111" s="10">
+      <c r="D111" s="9">
         <v>24405</v>
       </c>
-      <c r="E111" s="9" t="s">
+      <c r="E111" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F111" s="9" t="s">
+      <c r="F111" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="G111" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H111" s="9" t="s">
+      <c r="G111" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H111" s="8" t="s">
         <v>310</v>
       </c>
       <c r="I111" s="1"/>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A112" s="8">
-        <v>1</v>
-      </c>
-      <c r="B112" s="9" t="s">
+      <c r="A112" s="7">
+        <v>1</v>
+      </c>
+      <c r="B112" s="8" t="s">
         <v>238</v>
       </c>
-      <c r="C112" s="9" t="s">
+      <c r="C112" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="D112" s="10">
+      <c r="D112" s="9">
         <v>22598</v>
       </c>
-      <c r="E112" s="9" t="s">
+      <c r="E112" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="F112" s="9" t="s">
+      <c r="F112" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="G112" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H112" s="9" t="s">
+      <c r="G112" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H112" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I112" s="1"/>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A113" s="8">
-        <v>1</v>
-      </c>
-      <c r="B113" s="9" t="s">
+      <c r="A113" s="7">
+        <v>1</v>
+      </c>
+      <c r="B113" s="8" t="s">
         <v>241</v>
       </c>
-      <c r="C113" s="9" t="s">
+      <c r="C113" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D113" s="10">
+      <c r="D113" s="9">
         <v>24103</v>
       </c>
-      <c r="E113" s="9" t="s">
+      <c r="E113" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F113" s="9" t="s">
+      <c r="F113" s="8" t="s">
         <v>242</v>
       </c>
-      <c r="G113" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H113" s="9" t="s">
+      <c r="G113" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H113" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I113" s="1"/>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A114" s="17">
-        <v>1</v>
-      </c>
-      <c r="B114" s="18" t="s">
+      <c r="A114" s="16">
+        <v>1</v>
+      </c>
+      <c r="B114" s="17" t="s">
         <v>243</v>
       </c>
-      <c r="C114" s="18" t="s">
+      <c r="C114" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D114" s="19">
+      <c r="D114" s="18">
         <v>27262</v>
       </c>
-      <c r="E114" s="18" t="s">
+      <c r="E114" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="F114" s="18" t="s">
+      <c r="F114" s="17" t="s">
         <v>244</v>
       </c>
-      <c r="G114" s="18" t="s">
+      <c r="G114" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H114" s="18" t="s">
+      <c r="H114" s="17" t="s">
         <v>309</v>
       </c>
       <c r="I114" s="1"/>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A115" s="7">
-        <f>SUBTOTAL(9,A2:A114)</f>
-        <v>96</v>
-      </c>
-      <c r="B115" s="7"/>
-      <c r="C115" s="7"/>
-      <c r="D115" s="7"/>
-      <c r="E115" s="7"/>
-      <c r="F115" s="7"/>
-      <c r="G115" s="7"/>
-      <c r="H115" s="7"/>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A137">
+        <f>SUBTOTAL(9,A2:A136)</f>
+        <v>113</v>
+      </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138">
-        <f>SUBTOTAL(9,A2:A137)</f>
-        <v>96</v>
+        <f>SUBTOTAL(9,A3:A113)</f>
+        <v>111</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A139">
-        <f>SUBTOTAL(9,A3:A113)</f>
-        <v>94</v>
+        <f>SUBTOTAL(9,A2:A138)</f>
+        <v>113</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A140">
-        <f>SUBTOTAL(9,A2:A139)</f>
-        <v>96</v>
+        <f>SUBTOTAL(9,A3:A113)</f>
+        <v>111</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141">
+        <f>SUBTOTAL(9,A2:A140)</f>
+        <v>113</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A142" s="6">
         <f>SUBTOTAL(9,A3:A113)</f>
-        <v>94</v>
-      </c>
-    </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A142">
-        <f>SUBTOTAL(9,A2:A141)</f>
-        <v>96</v>
+        <v>111</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A143" s="6">
-        <f>SUBTOTAL(9,A3:A113)</f>
-        <v>94</v>
+      <c r="A143">
+        <f>SUBTOTAL(9,A2:A142)</f>
+        <v>113</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144">
-        <f>SUBTOTAL(9,A2:A143)</f>
-        <v>96</v>
-      </c>
-    </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A145">
         <f>SUBTOTAL(9,A3:A113)</f>
-        <v>94</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H114" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="7">
-      <filters>
-        <filter val="Valido"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:H114" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>